<commit_message>
Implement sync hardening and update docs/build
</commit_message>
<xml_diff>
--- a/lotto_history_20260204_132356.xlsx
+++ b/lotto_history_20260204_132356.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1209"/>
+  <dimension ref="A1:L1220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -48838,6 +48838,446 @@
         <v>62020198406</v>
       </c>
     </row>
+    <row r="1210">
+      <c r="A1210" s="2" t="n">
+        <v>1210</v>
+      </c>
+      <c r="B1210" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-07</t>
+        </is>
+      </c>
+      <c r="C1210" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1210" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E1210" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1210" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="G1210" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H1210" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="I1210" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="J1210" s="3" t="n">
+        <v>1102298407</v>
+      </c>
+      <c r="K1210" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="L1210" s="3" t="n">
+        <v>61555530677</v>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" s="2" t="n">
+        <v>1211</v>
+      </c>
+      <c r="B1211" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-14</t>
+        </is>
+      </c>
+      <c r="C1211" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="D1211" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="E1211" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="F1211" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G1211" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="H1211" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="I1211" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="J1211" s="3" t="n">
+        <v>2370956036</v>
+      </c>
+      <c r="K1211" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="L1211" s="3" t="n">
+        <v>67472903182</v>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" s="2" t="n">
+        <v>1212</v>
+      </c>
+      <c r="B1212" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-21</t>
+        </is>
+      </c>
+      <c r="C1212" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1212" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E1212" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F1212" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="G1212" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="H1212" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="I1212" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="J1212" s="3" t="n">
+        <v>2654089032</v>
+      </c>
+      <c r="K1212" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L1212" s="3" t="n">
+        <v>65863966662</v>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" s="2" t="n">
+        <v>1213</v>
+      </c>
+      <c r="B1213" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="C1213" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D1213" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E1213" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F1213" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1213" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="H1213" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="I1213" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J1213" s="3" t="n">
+        <v>1740011646</v>
+      </c>
+      <c r="K1213" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="L1213" s="3" t="n">
+        <v>65555539740</v>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" s="2" t="n">
+        <v>1214</v>
+      </c>
+      <c r="B1214" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="C1214" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D1214" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E1214" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="F1214" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1214" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="H1214" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="I1214" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="J1214" s="3" t="n">
+        <v>2431577188</v>
+      </c>
+      <c r="K1214" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L1214" s="3" t="n">
+        <v>62407932092</v>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" s="2" t="n">
+        <v>1215</v>
+      </c>
+      <c r="B1215" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-14</t>
+        </is>
+      </c>
+      <c r="C1215" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="D1215" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E1215" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="F1215" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="G1215" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="H1215" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="I1215" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="J1215" s="3" t="n">
+        <v>1998542133</v>
+      </c>
+      <c r="K1215" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="L1215" s="3" t="n">
+        <v>63488551584</v>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" s="2" t="n">
+        <v>1216</v>
+      </c>
+      <c r="B1216" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
+        </is>
+      </c>
+      <c r="C1216" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1216" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1216" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F1216" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="G1216" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="H1216" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="I1216" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="J1216" s="3" t="n">
+        <v>2148654000</v>
+      </c>
+      <c r="K1216" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="L1216" s="3" t="n">
+        <v>62778263417</v>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" s="2" t="n">
+        <v>1217</v>
+      </c>
+      <c r="B1217" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-28</t>
+        </is>
+      </c>
+      <c r="C1217" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D1217" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E1217" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F1217" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="G1217" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="H1217" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="I1217" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="J1217" s="3" t="n">
+        <v>2179738018</v>
+      </c>
+      <c r="K1217" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="L1217" s="3" t="n">
+        <v>62577629462</v>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" s="2" t="n">
+        <v>1218</v>
+      </c>
+      <c r="B1218" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-04</t>
+        </is>
+      </c>
+      <c r="C1218" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1218" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="E1218" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="F1218" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="G1218" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="H1218" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="I1218" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="J1218" s="3" t="n">
+        <v>1714482042</v>
+      </c>
+      <c r="K1218" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="L1218" s="3" t="n">
+        <v>61667966400</v>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" s="2" t="n">
+        <v>1219</v>
+      </c>
+      <c r="B1219" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-11</t>
+        </is>
+      </c>
+      <c r="C1219" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1219" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E1219" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F1219" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1219" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="H1219" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="I1219" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="J1219" s="3" t="n">
+        <v>2508232844</v>
+      </c>
+      <c r="K1219" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="L1219" s="3" t="n">
+        <v>60472901798</v>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" s="2" t="n">
+        <v>1220</v>
+      </c>
+      <c r="B1220" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="C1220" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1220" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="E1220" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F1220" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1220" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H1220" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="I1220" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="J1220" s="3" t="n">
+        <v>2114514161</v>
+      </c>
+      <c r="K1220" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="L1220" s="3" t="n">
+        <v>60979412665</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>